<commit_message>
fixed values in input file
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_earth_dam_rapid.xlsx
+++ b/docs/lem/files/xslope_earth_dam_rapid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCFABCD0-7B08-364D-AAB9-18954B999FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE96913C-38CC-FB4C-AC88-12A40BC83043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28360" yWindow="2300" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="4880" yWindow="3380" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1092,13 +1092,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -9743,10 +9743,10 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J10" s="3">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>89</v>
@@ -9804,7 +9804,7 @@
         <v>100</v>
       </c>
       <c r="J11" s="3">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>89</v>
@@ -10564,74 +10564,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="D4" s="46" t="s">
+      <c r="B4" s="48"/>
+      <c r="D4" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="G4" s="46" t="s">
+      <c r="E4" s="48"/>
+      <c r="G4" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="46"/>
-      <c r="J4" s="46" t="s">
+      <c r="H4" s="48"/>
+      <c r="J4" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="46"/>
-      <c r="M4" s="46" t="s">
+      <c r="K4" s="48"/>
+      <c r="M4" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="46"/>
-      <c r="P4" s="46" t="s">
+      <c r="N4" s="48"/>
+      <c r="P4" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="46"/>
+      <c r="Q4" s="48"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="46" t="s">
+      <c r="S4" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="46"/>
+      <c r="T4" s="48"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="46" t="s">
+      <c r="V4" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="46"/>
+      <c r="W4" s="48"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="46" t="s">
+      <c r="Y4" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="46"/>
+      <c r="Z4" s="48"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="46" t="s">
+      <c r="AB4" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="46"/>
-      <c r="AE4" s="46" t="s">
+      <c r="AC4" s="48"/>
+      <c r="AE4" s="48" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="46"/>
+      <c r="AF4" s="48"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="46" t="s">
+      <c r="AH4" s="48" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="46"/>
+      <c r="AI4" s="48"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="46" t="s">
+      <c r="AK4" s="48" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="46"/>
+      <c r="AL4" s="48"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="46" t="s">
+      <c r="AN4" s="48" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="46"/>
+      <c r="AO4" s="48"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="46" t="s">
+      <c r="AQ4" s="48" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="46"/>
+      <c r="AR4" s="48"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -10734,89 +10734,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="47" t="str">
+      <c r="A6" s="46" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Shell</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="D6" s="47" t="str">
+      <c r="B6" s="47"/>
+      <c r="D6" s="46" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Core</v>
       </c>
-      <c r="E6" s="48"/>
-      <c r="G6" s="47" t="str">
+      <c r="E6" s="47"/>
+      <c r="G6" s="46" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Clay</v>
       </c>
-      <c r="H6" s="48"/>
-      <c r="J6" s="47" t="str">
+      <c r="H6" s="47"/>
+      <c r="J6" s="46" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Sand</v>
       </c>
-      <c r="K6" s="48"/>
-      <c r="M6" s="47" t="str">
+      <c r="K6" s="47"/>
+      <c r="M6" s="46" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="48"/>
-      <c r="P6" s="47" t="str">
+      <c r="N6" s="47"/>
+      <c r="P6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="48"/>
+      <c r="Q6" s="47"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="47" t="str">
+      <c r="S6" s="46" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="48"/>
+      <c r="T6" s="47"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="47" t="str">
+      <c r="V6" s="46" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="48"/>
+      <c r="W6" s="47"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="47" t="str">
+      <c r="Y6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="48"/>
+      <c r="Z6" s="47"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="47" t="str">
+      <c r="AB6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="48"/>
-      <c r="AE6" s="47" t="str">
+      <c r="AC6" s="47"/>
+      <c r="AE6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="48"/>
+      <c r="AF6" s="47"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="47" t="str">
+      <c r="AH6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="48"/>
+      <c r="AI6" s="47"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="47" t="str">
+      <c r="AK6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="48"/>
+      <c r="AL6" s="47"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="47" t="str">
+      <c r="AN6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="48"/>
+      <c r="AO6" s="47"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="47" t="str">
+      <c r="AQ6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="48"/>
+      <c r="AR6" s="47"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11768,36 +11768,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>